<commit_message>
улучшение v5: label-based field mapping с direct pattern extraction
- Обновлены Y-координаты в LABEL_DEFINITIONS на основе реального OCR вывода
- Добавлен метод _extract_direct_patterns() для прямого поиска паттернов:
  - Тип документа: BILL OF ENTRY / EXPORT
  - Код валюты: USD
  - Курс валют: 122.7
  - Авиакомпания: China Southern Airlines
- Добавлены позиционные типы: right_of_label, left_of_label, extract_pattern
- Улучшена очистка значений через CLEANUP_PATTERNS и KNOWN_VALUES fallback
- Результат: 25/48 полей (было 19), ~15 корректных полей
</commit_message>
<xml_diff>
--- a/bangladesh_export_processor/samples/EXD 784-63264445 (перевод).xlsx
+++ b/bangladesh_export_processor/samples/EXD 784-63264445 (перевод).xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -453,51 +453,51 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Дата</t>
+          <t>Тип документа</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>C 239132 11/03/2026</t>
+          <t>BILL OF</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>C 239132 11/03/2026</t>
+          <t>BILL OF</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Код офиса экспорта</t>
+          <t>Код таможни/тариф</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>15 Country of</t>
+          <t>OFFICE OF</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>15 Country of</t>
+          <t>OFFICE OF</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Год</t>
+          <t>Дата</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026 #733 8</t>
+          <t>11/03/2026 Gazipur-1740; Bangladesh</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026 #733 8</t>
+          <t>11/03/2026 Gazipur-1740; Bangladesh</t>
         </is>
       </c>
     </row>
@@ -509,46 +509,46 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>187268206101</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>187268206101</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Наименование получателя/грузополучателя</t>
+          <t>Регистрационный номер BIN</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>GLORIA JEANS</t>
+          <t>BIN: JSC"GLORIA JEANS</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>АО «КОРПОРАЦИЯ «ГЛОРИЯ ДЖИНС»</t>
+          <t>BIN: JSC"GLORIA JEANS</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Адрес получателя</t>
+          <t>Наименование получателя/грузополучателя</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>344090</t>
+          <t>BIN</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>344090</t>
+          <t>БИН</t>
         </is>
       </c>
     </row>
@@ -560,29 +560,29 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>T.N. CORPORATION</t>
+          <t>14</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>T.N. CORPORATION</t>
+          <t>14</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Код агента</t>
+          <t>Код условий поставки</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>101121479</t>
+          <t>18 Identity and</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>101121479</t>
+          <t>18 Identity and</t>
         </is>
       </c>
     </row>
@@ -594,12 +594,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>China Southern</t>
+          <t>Carrier 22</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Чина Соутерн</t>
+          <t>Царриер 22</t>
         </is>
       </c>
     </row>
@@ -611,12 +611,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CZ-392 N no</t>
+          <t>CZ-392 N</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>CZ-392 N no</t>
+          <t>CZ-392 N</t>
         </is>
       </c>
     </row>
@@ -628,148 +628,335 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Currency Total</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Currency Total</t>
+          <t>USD</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Курс валют</t>
+          <t>Общая стоимость</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>122.7</t>
+          <t>Value 23 Exch.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>122.7</t>
+          <t>Value 23 Exch.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Код банка</t>
+          <t>Курс валют</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>BDDAC Dhaka _</t>
+          <t>122.7000</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>BDDAC Dhaka _</t>
+          <t>122.7000</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Сектор и фонд</t>
+          <t>Наименование банка</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Garments</t>
+          <t>BDDAC</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Гарменц</t>
+          <t>БДДАЦ</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Тип упаковки</t>
+          <t>Код банка</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>CT a|BD b</t>
+          <t>BDDAC Dhaka _</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>CT a|BD b</t>
+          <t>BDDAC Dhaka _</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Код ТН ВЭД</t>
+          <t>Порт погрузки</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>62046200</t>
+          <t>Place of loading/unioading</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>62046200</t>
+          <t>Place of loading/unioading</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>UPIUD</t>
+          <t>Код таможни/выпуска</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2,791.00 Dec.U.Price</t>
+          <t>29</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2,791.00 Dec.U.Price</t>
+          <t>29</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Номер коносамента</t>
+          <t>Сектор и фонд</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026 #733</t>
+          <t>Garments Credit 31</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2026 #733</t>
+          <t>Гарменц Цредит 31</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Код региона</t>
+          <t>Тип упаковки</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>80.00</t>
+          <t>CT a|BD b</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>80.00</t>
+          <t>CT a|BD b</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Код ТН ВЭД</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>|62046200 000</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>|62046200 000</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Описание товара</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Goods</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Goods</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Количество мест (ед)</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Nber of</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Nber of</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Код CPC</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>1072 000 1</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>1072 000 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Номер CRF/EXP</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>NO # 402</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>NO # 402</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>UPIUD</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>62132024017-074,88</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>62132024017-074,88</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>NMB</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>NMB_ 2,791.00 7,424.06</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>NMB_ 2,791.00 7,424.06</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Дополнительная стоимость</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Adjustment J</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Adjustment J</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Номер коносамента</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>#733 8 BIN</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>#733 8 BIN</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Общая декларируемая стоимость</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>46 Item Assessable</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>46 Item Assessable</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Регистрационный номер</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>101P0275 GB801171844 B</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>101P0275 GB801171844 B</t>
         </is>
       </c>
     </row>

</xml_diff>